<commit_message>
Plantillas de config.py iguales a ejemplos/config_*.json
- Insumos: bloques de 10:00 a 21:30, supermercados Unimarc reales
  (Irarrázaval, Príncipe de Gales, Los Militares) y nuevos pesos por bloque.
- Financiamiento: "Voluntario/a" también cuenta como jefe.
- Test que falla si config.py y los JSON de ejemplo dejan de coincidir.
- Respuestas ficticias de insumos regeneradas con los nuevos bloques y lugares.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019oe2a6HEDkUfhap1VckAWr
</commit_message>
<xml_diff>
--- a/ejemplos/respuestas_insumos_ficticias.xlsx
+++ b/ejemplos/respuestas_insumos_ficticias.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X61"/>
+  <dimension ref="A1:W61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,90 +449,85 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>¿Qué bloques puedes? [7:00 - 8:30]</t>
+          <t>¿Qué bloques puedes? [10:00 - 11:30]</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>¿Qué bloques puedes? [8:30 - 10:00]</t>
+          <t>¿Qué bloques puedes? [11:30 - 13:00]</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>¿Qué bloques puedes? [10:00 - 11:30]</t>
+          <t>¿Qué bloques puedes? [13:00 - 14:30]</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>¿Qué bloques puedes? [11:30 - 13:00]</t>
+          <t>¿Qué bloques puedes? [14:30 - 16:00]</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>¿Qué bloques puedes? [13:00 - 14:30]</t>
+          <t>¿Qué bloques puedes? [16:00 - 17:30]</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>¿Qué bloques puedes? [14:30 - 16:00]</t>
+          <t>¿Qué bloques puedes? [17:30 - 19:00]</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>¿Qué bloques puedes? [16:00 - 17:30]</t>
+          <t>¿Qué bloques puedes? [19:00 - 20:30]</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>¿Qué bloques puedes? [17:30 - 19:00]</t>
+          <t>¿Qué bloques puedes? [20:30 - 21:30]</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>¿Qué bloques puedes? [19:00 - 20:00]</t>
+          <t>¿Cuántos bloques como máximo por día? [Sábado]</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>¿Cuántos bloques como máximo por día? [Sábado]</t>
+          <t>¿Cuántos bloques como máximo por día? [Domingo]</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>¿Cuántos bloques como máximo por día? [Domingo]</t>
+          <t>¿En qué lugares puedes?</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>¿En qué lugares puedes?</t>
+          <t>¿Qué días tienes auto disponible?</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>¿Qué días tienes auto disponible?</t>
+          <t>¿Qué días puedes guardar insumos en tu casa?</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>¿Qué días puedes guardar insumos en tu casa?</t>
+          <t>Dirección donde guardarías los insumos</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>Dirección donde guardarías los insumos</t>
+          <t>Comuna</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>Comuna</t>
+          <t>Comentarios</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
-        <is>
-          <t>Comentarios</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
         <is>
           <t>¿Cuál es tu mood insumístico? (importantísimo)</t>
         </is>
@@ -572,45 +567,44 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Unimarc Los Militares, Unimarc Irarrázaval</t>
+        </is>
+      </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Supermercado Providencia, Supermercado Irarrázaval</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>A granel</t>
         </is>
@@ -671,32 +665,31 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Donde me necesiten</t>
+        </is>
+      </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>Enlatado</t>
         </is>
@@ -749,8 +742,7 @@
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>En oferta</t>
         </is>
@@ -808,31 +800,30 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Sin límite</t>
+        </is>
+      </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>Vencido</t>
         </is>
@@ -870,10 +861,14 @@
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado, Domingo</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -896,29 +891,25 @@
           <t>Sábado</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>2</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Sin límite</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>Unimarc Irarrázaval</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Supermercado Irarrázaval</t>
+          <t>Sábado, Domingo</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -928,21 +919,16 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
+          <t>Av. Los Leones 1500, Providencia</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Av. Los Leones 1500, Providencia</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
           <t>Providencia</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr">
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
         <is>
           <t>En oferta</t>
         </is>
@@ -982,45 +968,44 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Unimarc Los Militares, Unimarc Príncipe de Gales</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Supermercado Providencia, Supermercado Grecia</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>En oferta</t>
         </is>
@@ -1078,31 +1063,30 @@
       </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Unimarc Los Militares, Unimarc Príncipe de Gales</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Supermercado Providencia, Supermercado Grecia</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>Congelado</t>
         </is>
@@ -1168,31 +1152,30 @@
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>Vencido</t>
         </is>
@@ -1229,76 +1212,75 @@
           <t>Sí, voy con todo 🛒</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>2</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Unimarc Príncipe de Gales</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Supermercado Irarrázaval</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>En oferta</t>
         </is>
@@ -1327,34 +1309,73 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>No, odio a insumos 😔</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+          <t>Sí, voy con todo 🛒</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Sin límite</t>
+        </is>
+      </c>
       <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Unimarc Príncipe de Gales, Unimarc Los Militares</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>No tengo auto</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>No puedo</t>
+        </is>
+      </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>Congelado</t>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>A granel</t>
         </is>
       </c>
     </row>
@@ -1391,52 +1412,67 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Supermercado Grecia, Supermercado Providencia</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>No puedo</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr"/>
+          <t>Av. Grecia 1800, Ñuñoa</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Ñuñoa</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr">
-        <is>
-          <t>En oferta</t>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Congelado</t>
         </is>
       </c>
     </row>
@@ -1468,65 +1504,28 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Sí, voy con todo 🛒</t>
+          <t>No, odio a insumos 😔</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>Donde me necesiten</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>No puedo</t>
-        </is>
-      </c>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr">
-        <is>
-          <t>Congelado</t>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Vencido</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1552,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Comisionadx</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1562,7 +1561,11 @@
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>Domingo</t>
@@ -1578,49 +1581,36 @@
           <t>Domingo</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Unimarc Los Militares, Unimarc Irarrázaval</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr">
-        <is>
-          <t>Enlatado</t>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Vencido</t>
         </is>
       </c>
     </row>
@@ -1656,53 +1646,60 @@
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr"/>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>Unimarc Príncipe de Gales, Unimarc Irarrázaval, Unimarc Los Militares</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>En oferta</t>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Vencido</t>
         </is>
       </c>
     </row>
@@ -1729,7 +1726,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Comisionadx</t>
+          <t>Familia</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1740,59 +1737,54 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Sábado, Domingo</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Sábado, Domingo</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Supermercado Providencia, Supermercado Irarrázaval</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>Av. Irarrázaval 2900, Ñuñoa</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>Ñuñoa</t>
-        </is>
-      </c>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr">
-        <is>
-          <t>A granel</t>
+          <t>No puedo</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Congelado</t>
         </is>
       </c>
     </row>
@@ -1824,65 +1816,28 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Sí, voy con todo 🛒</t>
+          <t>No, odio a insumos 😔</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>Sin límite</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>Supermercado Grecia, Supermercado Providencia</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>No puedo</t>
-        </is>
-      </c>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr">
-        <is>
-          <t>Aplastado</t>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>A granel</t>
         </is>
       </c>
     </row>
@@ -1914,61 +1869,28 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Sí, voy con todo 🛒</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+          <t>No, odio a insumos 😔</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>Supermercado Irarrázaval, Supermercado Grecia, Supermercado Providencia</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>No puedo</t>
-        </is>
-      </c>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr">
-        <is>
-          <t>Aplastado</t>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>En oferta</t>
         </is>
       </c>
     </row>
@@ -1995,7 +1917,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2004,7 +1926,11 @@
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>Domingo</t>
@@ -2015,38 +1941,49 @@
           <t>Domingo</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Supermercado Irarrázaval, Supermercado Grecia</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>Vencido</t>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Congelado</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2010,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Familia</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2081,10 +2018,26 @@
           <t>Sí, voy con todo 🛒</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Sábado, Domingo</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Sábado, Domingo</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Sábado, Domingo</t>
+        </is>
+      </c>
       <c r="K20" t="inlineStr">
         <is>
           <t>Domingo</t>
@@ -2097,34 +2050,37 @@
       </c>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Unimarc Los Militares, Unimarc Irarrázaval, Unimarc Príncipe de Gales</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Supermercado Irarrázaval, Supermercado Providencia</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr">
-        <is>
-          <t>En oferta</t>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>Aplastado</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2107,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Comisionadx</t>
+          <t>Jefx de insumos</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2161,27 +2117,27 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Sábado, Domingo</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Sábado, Domingo</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Sábado, Domingo</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2189,44 +2145,43 @@
           <t>Sábado</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="P21" t="inlineStr">
         <is>
           <t>Sin límite</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Unimarc Príncipe de Gales, Unimarc Los Militares</t>
+        </is>
+      </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Supermercado Irarrázaval, Supermercado Providencia, Supermercado Grecia</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>Av. Grecia 1800, Ñuñoa</t>
-        </is>
-      </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>Ñuñoa</t>
-        </is>
-      </c>
-      <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr">
-        <is>
-          <t>En oferta</t>
+          <t>No puedo</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>Aplastado</t>
         </is>
       </c>
     </row>
@@ -2261,17 +2216,29 @@
           <t>Sí, voy con todo 🛒</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Sábado, Domingo</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Sábado, Domingo</t>
+        </is>
+      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Sábado, Domingo</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Sábado, Domingo</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2284,25 +2251,25 @@
           <t>Sábado</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>1</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr"/>
+          <t>Sin límite</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Unimarc Irarrázaval, Unimarc Los Militares, Unimarc Príncipe de Gales</t>
+        </is>
+      </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2312,13 +2279,16 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>No puedo</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr"/>
+          <t>Av. Los Leones 1500, Providencia</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Providencia</t>
+        </is>
+      </c>
       <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
-      <c r="X22" t="inlineStr">
+      <c r="W22" t="inlineStr">
         <is>
           <t>Enlatado</t>
         </is>
@@ -2355,36 +2325,40 @@
           <t>Sí, voy con todo 🛒</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2394,15 +2368,18 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>No puedo</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr"/>
+          <t>José Pedro Alessandri 1200, Ñuñoa</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Ñuñoa</t>
+        </is>
+      </c>
       <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
-      <c r="X23" t="inlineStr">
-        <is>
-          <t>Enlatado</t>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>Congelado</t>
         </is>
       </c>
     </row>
@@ -2429,34 +2406,77 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Familia</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>No, odio a insumos 😔</t>
+          <t>Sí, voy con todo 🛒</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Unimarc Príncipe de Gales</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>No tengo auto</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Av. Grecia 1800, Ñuñoa</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Ñuñoa</t>
+        </is>
+      </c>
       <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr">
-        <is>
-          <t>Vencido</t>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>Congelado</t>
         </is>
       </c>
     </row>
@@ -2492,75 +2512,58 @@
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Unimarc Príncipe de Gales, Unimarc Los Militares</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Supermercado Grecia, Supermercado Providencia</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25" t="inlineStr">
+      <c r="W25" t="inlineStr">
         <is>
           <t>Congelado</t>
         </is>
@@ -2602,34 +2605,30 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>Sábado, Domingo</t>
-        </is>
-      </c>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
           <t>3</t>
@@ -2637,30 +2636,33 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Unimarc Los Militares, Unimarc Irarrázaval</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Supermercado Grecia</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>No puedo</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr"/>
+          <t>Av. Pedro de Valdivia 3000, Providencia</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Providencia</t>
+        </is>
+      </c>
       <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr"/>
-      <c r="X26" t="inlineStr">
-        <is>
-          <t>Vencido</t>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>En oferta</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2689,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Comisionadx</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2696,61 +2698,64 @@
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr"/>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>Av. Grecia 1800, Ñuñoa</t>
-        </is>
-      </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>Ñuñoa</t>
-        </is>
-      </c>
-      <c r="W27" t="inlineStr"/>
-      <c r="X27" t="inlineStr">
-        <is>
-          <t>Congelado</t>
+          <t>No puedo</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>En oferta</t>
         </is>
       </c>
     </row>
@@ -2782,65 +2787,28 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Sí, voy con todo 🛒</t>
+          <t>No, odio a insumos 😔</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>Supermercado Irarrázaval, Supermercado Grecia, Supermercado Providencia</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>No puedo</t>
-        </is>
-      </c>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
-      <c r="X28" t="inlineStr">
-        <is>
-          <t>A granel</t>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>En oferta</t>
         </is>
       </c>
     </row>
@@ -2877,52 +2845,59 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Sin límite</t>
-        </is>
-      </c>
-      <c r="Q29" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Unimarc Los Militares, Unimarc Irarrázaval</t>
+        </is>
+      </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr"/>
-      <c r="X29" t="inlineStr">
-        <is>
-          <t>Aplastado</t>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>A granel</t>
         </is>
       </c>
     </row>
@@ -2960,59 +2935,58 @@
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>No puedo</t>
-        </is>
-      </c>
-      <c r="U30" t="inlineStr"/>
+          <t>Av. Pedro de Valdivia 3000, Providencia</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Providencia</t>
+        </is>
+      </c>
       <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr"/>
-      <c r="X30" t="inlineStr">
-        <is>
-          <t>A granel</t>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>Aplastado</t>
         </is>
       </c>
     </row>
@@ -3039,7 +3013,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Comisionadx</t>
+          <t>Familia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3047,62 +3021,73 @@
           <t>Sí, voy con todo 🛒</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Unimarc Príncipe de Gales, Unimarc Los Militares, Unimarc Irarrázaval</t>
+        </is>
+      </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>Supermercado Grecia, Supermercado Providencia</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>Av. Macul 3500, Macul</t>
-        </is>
-      </c>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>Macul</t>
-        </is>
-      </c>
-      <c r="W31" t="inlineStr"/>
-      <c r="X31" t="inlineStr">
-        <is>
-          <t>Congelado</t>
+          <t>No puedo</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>A granel</t>
         </is>
       </c>
     </row>
@@ -3129,7 +3114,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Familia</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3138,7 +3123,11 @@
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
           <t>Sábado</t>
@@ -3151,48 +3140,51 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
+          <t>Sábado, Domingo</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Sábado, Domingo</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Unimarc Príncipe de Gales, Unimarc Irarrázaval, Unimarc Los Militares</t>
+        </is>
+      </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>José Pedro Alessandri 1200, Ñuñoa</t>
-        </is>
-      </c>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>Ñuñoa</t>
-        </is>
-      </c>
-      <c r="W32" t="inlineStr"/>
-      <c r="X32" t="inlineStr">
-        <is>
-          <t>Enlatado</t>
+          <t>No puedo</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>A granel</t>
         </is>
       </c>
     </row>
@@ -3227,74 +3219,77 @@
           <t>Sí, voy con todo 🛒</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
           <t>Sábado, Domingo</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>Sábado, Domingo</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>Sábado, Domingo</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>Sábado, Domingo</t>
-        </is>
-      </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr"/>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>Unimarc Los Militares, Unimarc Irarrázaval, Unimarc Príncipe de Gales</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T33" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr"/>
-      <c r="W33" t="inlineStr"/>
-      <c r="X33" t="inlineStr">
-        <is>
-          <t>Aplastado</t>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>A granel</t>
         </is>
       </c>
     </row>
@@ -3321,7 +3316,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Comisionadx</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -3330,53 +3325,80 @@
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Unimarc Irarrázaval</t>
+        </is>
+      </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Supermercado Irarrázaval, Supermercado Providencia, Supermercado Grecia</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>No puedo</t>
-        </is>
-      </c>
-      <c r="U34" t="inlineStr"/>
+          <t>Av. Pedro de Valdivia 3000, Providencia</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Providencia</t>
+        </is>
+      </c>
       <c r="V34" t="inlineStr"/>
-      <c r="W34" t="inlineStr"/>
-      <c r="X34" t="inlineStr">
-        <is>
-          <t>Congelado</t>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>Aplastado</t>
         </is>
       </c>
     </row>
@@ -3403,7 +3425,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Familia</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3413,17 +3435,17 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="J35" t="inlineStr"/>
@@ -3434,35 +3456,30 @@
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="T35" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T35" t="inlineStr"/>
       <c r="U35" t="inlineStr"/>
       <c r="V35" t="inlineStr"/>
-      <c r="W35" t="inlineStr"/>
-      <c r="X35" t="inlineStr">
-        <is>
-          <t>Vencido</t>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>Congelado</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3506,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Jefx de insumos</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -3498,19 +3515,15 @@
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Sábado, Domingo</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -3520,33 +3533,37 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr"/>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -3556,23 +3573,18 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Av. Macul 3500, Macul</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>Av. Macul 3500, Macul</t>
-        </is>
-      </c>
-      <c r="V36" t="inlineStr">
-        <is>
           <t>Macul</t>
         </is>
       </c>
-      <c r="W36" t="inlineStr"/>
-      <c r="X36" t="inlineStr">
-        <is>
-          <t>Vencido</t>
+      <c r="V36" t="inlineStr"/>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>Aplastado</t>
         </is>
       </c>
     </row>
@@ -3631,36 +3643,35 @@
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Unimarc Irarrázaval</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Supermercado Irarrázaval</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="T37" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T37" t="inlineStr"/>
       <c r="U37" t="inlineStr"/>
       <c r="V37" t="inlineStr"/>
-      <c r="W37" t="inlineStr"/>
-      <c r="X37" t="inlineStr">
+      <c r="W37" t="inlineStr">
         <is>
           <t>En oferta</t>
         </is>
@@ -3700,45 +3711,44 @@
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="P38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Sin límite</t>
+        </is>
+      </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="T38" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T38" t="inlineStr"/>
       <c r="U38" t="inlineStr"/>
       <c r="V38" t="inlineStr"/>
-      <c r="W38" t="inlineStr"/>
-      <c r="X38" t="inlineStr">
+      <c r="W38" t="inlineStr">
         <is>
           <t>Aplastado</t>
         </is>
@@ -3811,36 +3821,35 @@
         </is>
       </c>
       <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Sin límite</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>Unimarc Los Militares, Unimarc Irarrázaval</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Supermercado Providencia, Supermercado Irarrázaval</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T39" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T39" t="inlineStr"/>
       <c r="U39" t="inlineStr"/>
       <c r="V39" t="inlineStr"/>
-      <c r="W39" t="inlineStr"/>
-      <c r="X39" t="inlineStr">
+      <c r="W39" t="inlineStr">
         <is>
           <t>A granel</t>
         </is>
@@ -3879,7 +3888,11 @@
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="J40" t="inlineStr">
         <is>
           <t>Sábado</t>
@@ -3907,34 +3920,29 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="P40" t="inlineStr">
-        <is>
           <t>Sin límite</t>
         </is>
       </c>
-      <c r="Q40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Unimarc Príncipe de Gales, Unimarc Los Militares, Unimarc Irarrázaval</t>
+        </is>
+      </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Supermercado Grecia, Supermercado Providencia</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T40" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T40" t="inlineStr"/>
       <c r="U40" t="inlineStr"/>
       <c r="V40" t="inlineStr"/>
-      <c r="W40" t="inlineStr"/>
-      <c r="X40" t="inlineStr">
+      <c r="W40" t="inlineStr">
         <is>
           <t>Enlatado</t>
         </is>
@@ -3987,8 +3995,7 @@
       <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr"/>
       <c r="V41" t="inlineStr"/>
-      <c r="W41" t="inlineStr"/>
-      <c r="X41" t="inlineStr">
+      <c r="W41" t="inlineStr">
         <is>
           <t>En oferta</t>
         </is>
@@ -4025,15 +4032,19 @@
           <t>Sí, voy con todo 🛒</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Sábado, Domingo</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -4056,53 +4067,44 @@
           <t>Domingo</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+      <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sin límite</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Av. Macul 3500, Macul</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>Av. Macul 3500, Macul</t>
-        </is>
-      </c>
-      <c r="V42" t="inlineStr">
-        <is>
           <t>Macul</t>
         </is>
       </c>
-      <c r="W42" t="inlineStr"/>
-      <c r="X42" t="inlineStr">
+      <c r="V42" t="inlineStr"/>
+      <c r="W42" t="inlineStr">
         <is>
           <t>En oferta</t>
         </is>
@@ -4141,46 +4143,45 @@
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr">
+      <c r="O43" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Donde me necesiten</t>
+        </is>
+      </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T43" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr"/>
       <c r="V43" t="inlineStr"/>
-      <c r="W43" t="inlineStr"/>
-      <c r="X43" t="inlineStr">
+      <c r="W43" t="inlineStr">
         <is>
           <t>Congelado</t>
         </is>
@@ -4218,8 +4219,16 @@
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="J44" t="inlineStr">
         <is>
           <t>Domingo</t>
@@ -4242,27 +4251,27 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sin límite</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Unimarc Príncipe de Gales</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Supermercado Grecia</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -4272,21 +4281,16 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Av. Pedro de Valdivia 3000, Providencia</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>Av. Pedro de Valdivia 3000, Providencia</t>
-        </is>
-      </c>
-      <c r="V44" t="inlineStr">
-        <is>
           <t>Providencia</t>
         </is>
       </c>
-      <c r="W44" t="inlineStr"/>
-      <c r="X44" t="inlineStr">
+      <c r="V44" t="inlineStr"/>
+      <c r="W44" t="inlineStr">
         <is>
           <t>En oferta</t>
         </is>
@@ -4347,32 +4351,31 @@
           <t>Sábado</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr">
+      <c r="O45" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="Q45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Donde me necesiten</t>
+        </is>
+      </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T45" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T45" t="inlineStr"/>
       <c r="U45" t="inlineStr"/>
       <c r="V45" t="inlineStr"/>
-      <c r="W45" t="inlineStr"/>
-      <c r="X45" t="inlineStr">
+      <c r="W45" t="inlineStr">
         <is>
           <t>Enlatado</t>
         </is>
@@ -4429,32 +4432,31 @@
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr">
+      <c r="O46" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="Q46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Donde me necesiten</t>
+        </is>
+      </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T46" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T46" t="inlineStr"/>
       <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr"/>
-      <c r="W46" t="inlineStr"/>
-      <c r="X46" t="inlineStr">
+      <c r="W46" t="inlineStr">
         <is>
           <t>Enlatado</t>
         </is>
@@ -4527,44 +4529,43 @@
         </is>
       </c>
       <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Unimarc Irarrázaval, Unimarc Príncipe de Gales</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>Supermercado Irarrázaval, Supermercado Grecia</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Av. Macul 3500, Macul</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>Av. Macul 3500, Macul</t>
-        </is>
-      </c>
-      <c r="V47" t="inlineStr">
-        <is>
           <t>Macul</t>
         </is>
       </c>
-      <c r="W47" t="inlineStr"/>
-      <c r="X47" t="inlineStr">
+      <c r="V47" t="inlineStr"/>
+      <c r="W47" t="inlineStr">
         <is>
           <t>Aplastado</t>
         </is>
@@ -4621,32 +4622,31 @@
         </is>
       </c>
       <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr">
+      <c r="O48" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="Q48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Unimarc Príncipe de Gales, Unimarc Los Militares</t>
+        </is>
+      </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>Supermercado Grecia, Supermercado Providencia</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T48" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T48" t="inlineStr"/>
       <c r="U48" t="inlineStr"/>
       <c r="V48" t="inlineStr"/>
-      <c r="W48" t="inlineStr"/>
-      <c r="X48" t="inlineStr">
+      <c r="W48" t="inlineStr">
         <is>
           <t>A granel</t>
         </is>
@@ -4704,39 +4704,38 @@
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Unimarc Los Militares, Unimarc Príncipe de Gales, Unimarc Irarrázaval</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>Supermercado Providencia, Supermercado Grecia, Supermercado Irarrázaval</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Av. Los Leones 1500, Providencia</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>Av. Los Leones 1500, Providencia</t>
-        </is>
-      </c>
-      <c r="V49" t="inlineStr">
-        <is>
           <t>Providencia</t>
         </is>
       </c>
-      <c r="W49" t="inlineStr"/>
-      <c r="X49" t="inlineStr">
+      <c r="V49" t="inlineStr"/>
+      <c r="W49" t="inlineStr">
         <is>
           <t>Congelado</t>
         </is>
@@ -4773,7 +4772,11 @@
           <t>Sí, voy con todo 🛒</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="H50" t="inlineStr">
         <is>
           <t>Sábado</t>
@@ -4801,40 +4804,39 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Sin límite</t>
+        </is>
+      </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="T50" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr"/>
       <c r="V50" t="inlineStr"/>
-      <c r="W50" t="inlineStr"/>
-      <c r="X50" t="inlineStr">
+      <c r="W50" t="inlineStr">
         <is>
           <t>Congelado</t>
         </is>
@@ -4899,36 +4901,35 @@
         </is>
       </c>
       <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Unimarc Irarrázaval, Unimarc Príncipe de Gales</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Supermercado Irarrázaval, Supermercado Grecia</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T51" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T51" t="inlineStr"/>
       <c r="U51" t="inlineStr"/>
       <c r="V51" t="inlineStr"/>
-      <c r="W51" t="inlineStr"/>
-      <c r="X51" t="inlineStr">
+      <c r="W51" t="inlineStr">
         <is>
           <t>A granel</t>
         </is>
@@ -4981,8 +4982,7 @@
       <c r="T52" t="inlineStr"/>
       <c r="U52" t="inlineStr"/>
       <c r="V52" t="inlineStr"/>
-      <c r="W52" t="inlineStr"/>
-      <c r="X52" t="inlineStr">
+      <c r="W52" t="inlineStr">
         <is>
           <t>Aplastado</t>
         </is>
@@ -5044,31 +5044,30 @@
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr"/>
       <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Sin límite</t>
+        </is>
+      </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>Unimarc Los Militares, Unimarc Irarrázaval</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>Supermercado Providencia, Supermercado Irarrázaval</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T53" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T53" t="inlineStr"/>
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr"/>
-      <c r="W53" t="inlineStr"/>
-      <c r="X53" t="inlineStr">
+      <c r="W53" t="inlineStr">
         <is>
           <t>En oferta</t>
         </is>
@@ -5137,36 +5136,35 @@
       </c>
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Sin límite</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="T54" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T54" t="inlineStr"/>
       <c r="U54" t="inlineStr"/>
       <c r="V54" t="inlineStr"/>
-      <c r="W54" t="inlineStr"/>
-      <c r="X54" t="inlineStr">
+      <c r="W54" t="inlineStr">
         <is>
           <t>Vencido</t>
         </is>
@@ -5227,32 +5225,31 @@
         </is>
       </c>
       <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr">
+      <c r="O55" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="Q55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>Donde me necesiten</t>
+        </is>
+      </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="T55" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T55" t="inlineStr"/>
       <c r="U55" t="inlineStr"/>
       <c r="V55" t="inlineStr"/>
-      <c r="W55" t="inlineStr"/>
-      <c r="X55" t="inlineStr">
+      <c r="W55" t="inlineStr">
         <is>
           <t>Aplastado</t>
         </is>
@@ -5290,28 +5287,32 @@
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+      <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>2</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -5321,36 +5322,31 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Unimarc Príncipe de Gales</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>Supermercado Grecia</t>
+          <t>Sábado, Domingo</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>Sábado, Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>José Pedro Alessandri 1200, Ñuñoa</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
         <is>
-          <t>José Pedro Alessandri 1200, Ñuñoa</t>
-        </is>
-      </c>
-      <c r="V56" t="inlineStr">
-        <is>
           <t>Ñuñoa</t>
         </is>
       </c>
-      <c r="W56" t="inlineStr"/>
-      <c r="X56" t="inlineStr">
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="inlineStr">
         <is>
           <t>Enlatado</t>
         </is>
@@ -5411,36 +5407,35 @@
       </c>
       <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Unimarc Los Militares</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>Supermercado Providencia</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="T57" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T57" t="inlineStr"/>
       <c r="U57" t="inlineStr"/>
       <c r="V57" t="inlineStr"/>
-      <c r="W57" t="inlineStr"/>
-      <c r="X57" t="inlineStr">
+      <c r="W57" t="inlineStr">
         <is>
           <t>Congelado</t>
         </is>
@@ -5502,15 +5497,19 @@
       <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr"/>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Unimarc Los Militares</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>Supermercado Providencia</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
@@ -5520,21 +5519,16 @@
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Av. Los Leones 1500, Providencia</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
         <is>
-          <t>Av. Los Leones 1500, Providencia</t>
-        </is>
-      </c>
-      <c r="V58" t="inlineStr">
-        <is>
           <t>Providencia</t>
         </is>
       </c>
-      <c r="W58" t="inlineStr"/>
-      <c r="X58" t="inlineStr">
+      <c r="V58" t="inlineStr"/>
+      <c r="W58" t="inlineStr">
         <is>
           <t>En oferta</t>
         </is>
@@ -5578,7 +5572,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Sábado, Domingo</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5606,41 +5600,36 @@
           <t>Domingo</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
-      <c r="O59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Sin límite</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="T59" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T59" t="inlineStr"/>
       <c r="U59" t="inlineStr"/>
       <c r="V59" t="inlineStr"/>
-      <c r="W59" t="inlineStr"/>
-      <c r="X59" t="inlineStr">
+      <c r="W59" t="inlineStr">
         <is>
           <t>Enlatado</t>
         </is>
@@ -5678,8 +5667,16 @@
         </is>
       </c>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="J60" t="inlineStr">
         <is>
           <t>Sábado</t>
@@ -5700,41 +5697,32 @@
           <t>Sábado</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="P60" t="inlineStr">
-        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="Q60" t="inlineStr"/>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Donde me necesiten</t>
+        </is>
+      </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T60" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T60" t="inlineStr"/>
       <c r="U60" t="inlineStr"/>
       <c r="V60" t="inlineStr"/>
-      <c r="W60" t="inlineStr"/>
-      <c r="X60" t="inlineStr">
+      <c r="W60" t="inlineStr">
         <is>
           <t>Vencido</t>
         </is>
@@ -5771,7 +5759,11 @@
           <t>Sí, voy con todo 🛒</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="H61" t="inlineStr">
         <is>
           <t>Sábado</t>
@@ -5797,38 +5789,33 @@
           <t>Sábado</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr">
+      <c r="O61" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="Q61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>Unimarc Los Militares, Unimarc Irarrázaval, Unimarc Príncipe de Gales</t>
+        </is>
+      </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>Supermercado Providencia, Supermercado Irarrázaval, Supermercado Grecia</t>
+          <t>No tengo auto</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>No tengo auto</t>
-        </is>
-      </c>
-      <c r="T61" t="inlineStr">
-        <is>
           <t>No puedo</t>
         </is>
       </c>
+      <c r="T61" t="inlineStr"/>
       <c r="U61" t="inlineStr"/>
       <c r="V61" t="inlineStr"/>
-      <c r="W61" t="inlineStr"/>
-      <c r="X61" t="inlineStr">
+      <c r="W61" t="inlineStr">
         <is>
           <t>En oferta</t>
         </is>

</xml_diff>